<commit_message>
updated with lookuph and lookupv
</commit_message>
<xml_diff>
--- a/batch_04/Basic_formulas.xlsx
+++ b/batch_04/Basic_formulas.xlsx
@@ -1,31 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TrainerDoc\Programming\data_analytics\batch_03\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\data_analytics\batch_04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D064DCB-F9D9-4574-AEC4-549CBD95DE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11640" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11640"/>
   </bookViews>
   <sheets>
-    <sheet name="Basic Math Formulas" sheetId="4" r:id="rId1"/>
-    <sheet name="date and Time Functions" sheetId="2" r:id="rId2"/>
-    <sheet name="Text Functins" sheetId="1" r:id="rId3"/>
-    <sheet name="Logical Functions" sheetId="3" r:id="rId4"/>
-    <sheet name="Statistical Functions" sheetId="5" r:id="rId5"/>
-    <sheet name="Lookup (V and H _Lookup) " sheetId="6" r:id="rId6"/>
-    <sheet name="Reference Functions" sheetId="7" r:id="rId7"/>
-    <sheet name="Sheet1" sheetId="8" r:id="rId8"/>
+    <sheet name="lookupH" sheetId="10" r:id="rId1"/>
+    <sheet name="LookupV" sheetId="9" r:id="rId2"/>
+    <sheet name="Basic Math Formulas" sheetId="4" r:id="rId3"/>
+    <sheet name="date and Time Functions" sheetId="2" r:id="rId4"/>
+    <sheet name="Text Functins" sheetId="1" r:id="rId5"/>
+    <sheet name="Logical Functions" sheetId="3" r:id="rId6"/>
+    <sheet name="Statistical Functions" sheetId="5" r:id="rId7"/>
+    <sheet name="Lookup (V and H _Lookup) " sheetId="6" r:id="rId8"/>
+    <sheet name="Reference Functions" sheetId="7" r:id="rId9"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Logical Functions'!$A$5:$G$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Logical Functions'!$A$5:$G$8</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="233">
   <si>
     <t>CONCATENATE(), TEXT(), LEFT(), RIGHT(), MID(), LEN(), TRIM(), UPPER(), LOWER(), PROPER(), REPT(), SUBSTITUTE(), FIND(), SEARCH()</t>
   </si>
@@ -646,12 +647,102 @@
   </si>
   <si>
     <t>python</t>
+  </si>
+  <si>
+    <t>RegNo</t>
+  </si>
+  <si>
+    <t>Student Name</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>cc</t>
+  </si>
+  <si>
+    <t>Paid</t>
+  </si>
+  <si>
+    <t>Balance</t>
+  </si>
+  <si>
+    <t>Arjun Kumar</t>
+  </si>
+  <si>
+    <t>Priya Sharma</t>
+  </si>
+  <si>
+    <t>Bangalore</t>
+  </si>
+  <si>
+    <t>Rahul Verma</t>
+  </si>
+  <si>
+    <t>Sneha Reddy</t>
+  </si>
+  <si>
+    <t>Coimbatore</t>
+  </si>
+  <si>
+    <t>Karthik Raj</t>
+  </si>
+  <si>
+    <t>Ananya Singh</t>
+  </si>
+  <si>
+    <t>Vishal Mehta</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>Divya Nair</t>
+  </si>
+  <si>
+    <t>Sanjay Patel</t>
+  </si>
+  <si>
+    <t>Ahmedabad</t>
+  </si>
+  <si>
+    <t>Meera Iyer</t>
+  </si>
+  <si>
+    <t>Rohit Das</t>
+  </si>
+  <si>
+    <t>Kavya Krishna</t>
+  </si>
+  <si>
+    <t>Aditya Rao</t>
+  </si>
+  <si>
+    <t>Lakshmi Priya</t>
+  </si>
+  <si>
+    <t>Salem</t>
+  </si>
+  <si>
+    <t>Naveen Kumar</t>
+  </si>
+  <si>
+    <t>Tirunelveli</t>
+  </si>
+  <si>
+    <t>Fees (₹)</t>
+  </si>
+  <si>
+    <t>Paid (₹)</t>
+  </si>
+  <si>
+    <t>Balance (₹)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000000"/>
   </numFmts>
@@ -805,7 +896,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -881,6 +972,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1198,7 +1292,928 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:P18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="28" t="s">
+        <v>203</v>
+      </c>
+      <c r="B1" s="30">
+        <v>101</v>
+      </c>
+      <c r="C1" s="30">
+        <v>102</v>
+      </c>
+      <c r="D1" s="30">
+        <v>102</v>
+      </c>
+      <c r="E1" s="30">
+        <v>102</v>
+      </c>
+      <c r="F1" s="30">
+        <v>105</v>
+      </c>
+      <c r="G1" s="30">
+        <v>106</v>
+      </c>
+      <c r="H1" s="30">
+        <v>107</v>
+      </c>
+      <c r="I1" s="30">
+        <v>108</v>
+      </c>
+      <c r="J1" s="30">
+        <v>109</v>
+      </c>
+      <c r="K1" s="30">
+        <v>110</v>
+      </c>
+      <c r="L1" s="30">
+        <v>111</v>
+      </c>
+      <c r="M1" s="30">
+        <v>112</v>
+      </c>
+      <c r="N1" s="30">
+        <v>113</v>
+      </c>
+      <c r="O1" s="30">
+        <v>114</v>
+      </c>
+      <c r="P1" s="30">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>209</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>210</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>212</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>213</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>215</v>
+      </c>
+      <c r="G2" s="30" t="s">
+        <v>216</v>
+      </c>
+      <c r="H2" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="I2" s="30" t="s">
+        <v>219</v>
+      </c>
+      <c r="J2" s="30" t="s">
+        <v>220</v>
+      </c>
+      <c r="K2" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="L2" s="30" t="s">
+        <v>223</v>
+      </c>
+      <c r="M2" s="30" t="s">
+        <v>224</v>
+      </c>
+      <c r="N2" s="30" t="s">
+        <v>225</v>
+      </c>
+      <c r="O2" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="P2" s="30" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="28" t="s">
+        <v>146</v>
+      </c>
+      <c r="B3" s="30">
+        <v>19</v>
+      </c>
+      <c r="C3" s="30">
+        <v>20</v>
+      </c>
+      <c r="D3" s="30">
+        <v>18</v>
+      </c>
+      <c r="E3" s="30">
+        <v>21</v>
+      </c>
+      <c r="F3" s="30">
+        <v>19</v>
+      </c>
+      <c r="G3" s="30">
+        <v>22</v>
+      </c>
+      <c r="H3" s="30">
+        <v>20</v>
+      </c>
+      <c r="I3" s="30">
+        <v>18</v>
+      </c>
+      <c r="J3" s="30">
+        <v>21</v>
+      </c>
+      <c r="K3" s="30">
+        <v>19</v>
+      </c>
+      <c r="L3" s="30">
+        <v>23</v>
+      </c>
+      <c r="M3" s="30">
+        <v>20</v>
+      </c>
+      <c r="N3" s="30">
+        <v>22</v>
+      </c>
+      <c r="O3" s="30">
+        <v>18</v>
+      </c>
+      <c r="P3" s="30">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="28" t="s">
+        <v>205</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>211</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>211</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>214</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>214</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>214</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>218</v>
+      </c>
+      <c r="I4" s="30" t="s">
+        <v>211</v>
+      </c>
+      <c r="J4" s="30" t="s">
+        <v>221</v>
+      </c>
+      <c r="K4" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="N4" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="O4" s="30" t="s">
+        <v>227</v>
+      </c>
+      <c r="P4" s="30" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
+        <v>230</v>
+      </c>
+      <c r="B5" s="30">
+        <v>50000</v>
+      </c>
+      <c r="C5" s="30">
+        <v>55000</v>
+      </c>
+      <c r="D5" s="30">
+        <v>48000</v>
+      </c>
+      <c r="E5" s="30">
+        <v>52000</v>
+      </c>
+      <c r="F5" s="30">
+        <v>47000</v>
+      </c>
+      <c r="G5" s="30">
+        <v>60000</v>
+      </c>
+      <c r="H5" s="30">
+        <v>58000</v>
+      </c>
+      <c r="I5" s="30">
+        <v>45000</v>
+      </c>
+      <c r="J5" s="30">
+        <v>53000</v>
+      </c>
+      <c r="K5" s="30">
+        <v>49000</v>
+      </c>
+      <c r="L5" s="30">
+        <v>61000</v>
+      </c>
+      <c r="M5" s="30">
+        <v>52000</v>
+      </c>
+      <c r="N5" s="30">
+        <v>57000</v>
+      </c>
+      <c r="O5" s="30">
+        <v>46000</v>
+      </c>
+      <c r="P5" s="30">
+        <v>54000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="28" t="s">
+        <v>231</v>
+      </c>
+      <c r="B6" s="30">
+        <v>30000</v>
+      </c>
+      <c r="C6" s="30">
+        <v>55000</v>
+      </c>
+      <c r="D6" s="30">
+        <v>20000</v>
+      </c>
+      <c r="E6" s="30">
+        <v>40000</v>
+      </c>
+      <c r="F6" s="30">
+        <v>47000</v>
+      </c>
+      <c r="G6" s="30">
+        <v>35000</v>
+      </c>
+      <c r="H6" s="30">
+        <v>30000</v>
+      </c>
+      <c r="I6" s="30">
+        <v>45000</v>
+      </c>
+      <c r="J6" s="30">
+        <v>25000</v>
+      </c>
+      <c r="K6" s="30">
+        <v>49000</v>
+      </c>
+      <c r="L6" s="30">
+        <v>40000</v>
+      </c>
+      <c r="M6" s="30">
+        <v>30000</v>
+      </c>
+      <c r="N6" s="30">
+        <v>20000</v>
+      </c>
+      <c r="O6" s="30">
+        <v>30000</v>
+      </c>
+      <c r="P6" s="30">
+        <v>54000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="28" t="s">
+        <v>232</v>
+      </c>
+      <c r="B7" s="30">
+        <v>20000</v>
+      </c>
+      <c r="C7" s="30">
+        <v>0</v>
+      </c>
+      <c r="D7" s="30">
+        <v>28000</v>
+      </c>
+      <c r="E7" s="30">
+        <v>12000</v>
+      </c>
+      <c r="F7" s="30">
+        <v>0</v>
+      </c>
+      <c r="G7" s="30">
+        <v>25000</v>
+      </c>
+      <c r="H7" s="30">
+        <v>28000</v>
+      </c>
+      <c r="I7" s="30">
+        <v>0</v>
+      </c>
+      <c r="J7" s="30">
+        <v>28000</v>
+      </c>
+      <c r="K7" s="30">
+        <v>0</v>
+      </c>
+      <c r="L7" s="30">
+        <v>21000</v>
+      </c>
+      <c r="M7" s="30">
+        <v>22000</v>
+      </c>
+      <c r="N7" s="30">
+        <v>37000</v>
+      </c>
+      <c r="O7" s="30">
+        <v>16000</v>
+      </c>
+      <c r="P7" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F17" t="s">
+        <v>209</v>
+      </c>
+      <c r="G17">
+        <f>HLOOKUP(F17,B2:P7,6,FALSE)</f>
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="18" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F18">
+        <v>105</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="str">
+        <f>'Reference Functions'!A4</f>
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <f>'Reference Functions'!C4</f>
+        <v>Gender</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>'Reference Functions'!A5</f>
+        <v>John</v>
+      </c>
+      <c r="B2" t="str">
+        <f>'Reference Functions'!C5</f>
+        <v>Male</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f>'Reference Functions'!A6</f>
+        <v>Sarah</v>
+      </c>
+      <c r="B3" t="str">
+        <f>'Reference Functions'!C6</f>
+        <v>Female</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f>'Reference Functions'!A7</f>
+        <v>Mike</v>
+      </c>
+      <c r="B4" t="str">
+        <f>'Reference Functions'!C7</f>
+        <v>male</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <f>'Reference Functions'!A8</f>
+        <v>0</v>
+      </c>
+      <c r="B5">
+        <f>'Reference Functions'!C8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <f>'Reference Functions'!A9</f>
+        <v>0</v>
+      </c>
+      <c r="B6">
+        <f>'Reference Functions'!C9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <f>'Reference Functions'!A10</f>
+        <v>0</v>
+      </c>
+      <c r="B7">
+        <f>'Reference Functions'!C10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <f>'Reference Functions'!A11</f>
+        <v>0</v>
+      </c>
+      <c r="B8">
+        <f>'Reference Functions'!C11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <f>'Reference Functions'!A12</f>
+        <v>0</v>
+      </c>
+      <c r="B9">
+        <f>'Reference Functions'!C12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <f>'Reference Functions'!A13</f>
+        <v>0</v>
+      </c>
+      <c r="B10">
+        <f>'Reference Functions'!C13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <f>'Reference Functions'!A14</f>
+        <v>0</v>
+      </c>
+      <c r="B11">
+        <f>'Reference Functions'!C14</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" customWidth="1"/>
+    <col min="11" max="11" width="16.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="37" t="s">
+        <v>203</v>
+      </c>
+      <c r="B1" s="37" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1" s="37" t="s">
+        <v>146</v>
+      </c>
+      <c r="D1" s="37" t="s">
+        <v>205</v>
+      </c>
+      <c r="E1" s="37" t="s">
+        <v>206</v>
+      </c>
+      <c r="F1" s="37" t="s">
+        <v>207</v>
+      </c>
+      <c r="G1" s="37" t="s">
+        <v>208</v>
+      </c>
+      <c r="K1">
+        <f>MATCH("Paid",A1:G1)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="27">
+        <v>101</v>
+      </c>
+      <c r="B2" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="C2" s="27">
+        <v>19</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="27">
+        <v>50000</v>
+      </c>
+      <c r="F2" s="27">
+        <v>30000</v>
+      </c>
+      <c r="G2" s="27">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="27">
+        <v>102</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="C3" s="27">
+        <v>20</v>
+      </c>
+      <c r="D3" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="E3" s="27">
+        <v>55000</v>
+      </c>
+      <c r="F3" s="27">
+        <v>55000</v>
+      </c>
+      <c r="G3" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="27">
+        <v>102</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="C4" s="27">
+        <v>18</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="E4" s="27">
+        <v>48000</v>
+      </c>
+      <c r="F4" s="27">
+        <v>20000</v>
+      </c>
+      <c r="G4" s="27">
+        <v>28000</v>
+      </c>
+      <c r="J4" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="K4">
+        <f>VLOOKUP(J4,B2:G16,MATCH(J10,A1:G1,),FALSE)</f>
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="27">
+        <v>102</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>213</v>
+      </c>
+      <c r="C5" s="27">
+        <v>21</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>214</v>
+      </c>
+      <c r="E5" s="27">
+        <v>52000</v>
+      </c>
+      <c r="F5" s="27">
+        <v>40000</v>
+      </c>
+      <c r="G5" s="27">
+        <v>12000</v>
+      </c>
+      <c r="J5" s="27">
+        <v>104</v>
+      </c>
+      <c r="K5">
+        <f>VLOOKUP(105,A2:G16,7,FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="27">
+        <v>105</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="C6" s="27">
+        <v>19</v>
+      </c>
+      <c r="D6" s="27" t="s">
+        <v>214</v>
+      </c>
+      <c r="E6" s="27">
+        <v>47000</v>
+      </c>
+      <c r="F6" s="27">
+        <v>47000</v>
+      </c>
+      <c r="G6" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="27">
+        <v>106</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>216</v>
+      </c>
+      <c r="C7" s="27">
+        <v>22</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>214</v>
+      </c>
+      <c r="E7" s="27">
+        <v>60000</v>
+      </c>
+      <c r="F7" s="27">
+        <v>35000</v>
+      </c>
+      <c r="G7" s="27">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="27">
+        <v>107</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="C8" s="27">
+        <v>20</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E8" s="27">
+        <v>58000</v>
+      </c>
+      <c r="F8" s="27">
+        <v>30000</v>
+      </c>
+      <c r="G8" s="27">
+        <v>28000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="27">
+        <v>108</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>219</v>
+      </c>
+      <c r="C9" s="27">
+        <v>18</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="E9" s="27">
+        <v>45000</v>
+      </c>
+      <c r="F9" s="27">
+        <v>45000</v>
+      </c>
+      <c r="G9" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="27">
+        <v>109</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="C10" s="27">
+        <v>21</v>
+      </c>
+      <c r="D10" s="27" t="s">
+        <v>221</v>
+      </c>
+      <c r="E10" s="27">
+        <v>53000</v>
+      </c>
+      <c r="F10" s="27">
+        <v>25000</v>
+      </c>
+      <c r="G10" s="27">
+        <v>28000</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="27">
+        <v>110</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>222</v>
+      </c>
+      <c r="C11" s="27">
+        <v>19</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="27">
+        <v>49000</v>
+      </c>
+      <c r="F11" s="27">
+        <v>49000</v>
+      </c>
+      <c r="G11" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="27">
+        <v>111</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="C12" s="27">
+        <v>23</v>
+      </c>
+      <c r="D12" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="27">
+        <v>61000</v>
+      </c>
+      <c r="F12" s="27">
+        <v>40000</v>
+      </c>
+      <c r="G12" s="27">
+        <v>21000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="27">
+        <v>112</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C13" s="27">
+        <v>20</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="27">
+        <v>52000</v>
+      </c>
+      <c r="F13" s="27">
+        <v>30000</v>
+      </c>
+      <c r="G13" s="27">
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="27">
+        <v>113</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>225</v>
+      </c>
+      <c r="C14" s="27">
+        <v>22</v>
+      </c>
+      <c r="D14" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="27">
+        <v>57000</v>
+      </c>
+      <c r="F14" s="27">
+        <v>20000</v>
+      </c>
+      <c r="G14" s="27">
+        <v>37000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="27">
+        <v>114</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="C15" s="27">
+        <v>18</v>
+      </c>
+      <c r="D15" s="27" t="s">
+        <v>227</v>
+      </c>
+      <c r="E15" s="27">
+        <v>46000</v>
+      </c>
+      <c r="F15" s="27">
+        <v>30000</v>
+      </c>
+      <c r="G15" s="27">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="27">
+        <v>115</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>228</v>
+      </c>
+      <c r="C16" s="27">
+        <v>21</v>
+      </c>
+      <c r="D16" s="27" t="s">
+        <v>229</v>
+      </c>
+      <c r="E16" s="27">
+        <v>54000</v>
+      </c>
+      <c r="F16" s="27">
+        <v>54000</v>
+      </c>
+      <c r="G16" s="27">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:R21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1342,11 +2357,11 @@
       </c>
       <c r="Q2" s="21">
         <f ca="1">RAND()</f>
-        <v>0.72901728750663719</v>
+        <v>0.34995558823598472</v>
       </c>
       <c r="R2" s="21">
         <f ca="1">RANDBETWEEN(1000,9999)</f>
-        <v>5953</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
@@ -1414,11 +2429,11 @@
       </c>
       <c r="Q3" s="21">
         <f t="shared" ref="Q3:Q10" ca="1" si="14">RAND()</f>
-        <v>0.66559471269613701</v>
+        <v>0.20688850921956303</v>
       </c>
       <c r="R3" s="21">
         <f ca="1">RANDBETWEEN(1000,9999)</f>
-        <v>1302</v>
+        <v>9953</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -1486,11 +2501,11 @@
       </c>
       <c r="Q4" s="21">
         <f t="shared" ca="1" si="14"/>
-        <v>0.20546439943359551</v>
+        <v>0.382879304507873</v>
       </c>
       <c r="R4" s="21">
         <f t="shared" ref="R4:R10" ca="1" si="15">RANDBETWEEN(1000,9999)</f>
-        <v>2452</v>
+        <v>6934</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -1558,11 +2573,11 @@
       </c>
       <c r="Q5" s="21">
         <f t="shared" ca="1" si="14"/>
-        <v>0.18027926433163421</v>
+        <v>0.45051492167902696</v>
       </c>
       <c r="R5" s="21">
         <f t="shared" ca="1" si="15"/>
-        <v>8666</v>
+        <v>4671</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -1630,11 +2645,11 @@
       </c>
       <c r="Q6" s="21">
         <f t="shared" ca="1" si="14"/>
-        <v>0.5800268124659097</v>
+        <v>0.31399391525938747</v>
       </c>
       <c r="R6" s="21">
         <f t="shared" ca="1" si="15"/>
-        <v>3129</v>
+        <v>8224</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
@@ -1702,11 +2717,11 @@
       </c>
       <c r="Q7" s="21">
         <f t="shared" ca="1" si="14"/>
-        <v>0.50979355468534504</v>
+        <v>2.7709531483813832E-3</v>
       </c>
       <c r="R7" s="21">
         <f t="shared" ca="1" si="15"/>
-        <v>7751</v>
+        <v>6065</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
@@ -1774,11 +2789,11 @@
       </c>
       <c r="Q8" s="21">
         <f t="shared" ca="1" si="14"/>
-        <v>0.36680329558310953</v>
+        <v>0.38990190176643946</v>
       </c>
       <c r="R8" s="21">
         <f t="shared" ca="1" si="15"/>
-        <v>3635</v>
+        <v>7650</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
@@ -1846,11 +2861,11 @@
       </c>
       <c r="Q9" s="21">
         <f t="shared" ca="1" si="14"/>
-        <v>0.12761270558447246</v>
+        <v>0.63928787831614808</v>
       </c>
       <c r="R9" s="21">
         <f t="shared" ca="1" si="15"/>
-        <v>3674</v>
+        <v>6435</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -1918,11 +2933,11 @@
       </c>
       <c r="Q10" s="21">
         <f t="shared" ca="1" si="14"/>
-        <v>0.18621938465794574</v>
+        <v>2.1642461985010408E-2</v>
       </c>
       <c r="R10" s="21">
         <f t="shared" ca="1" si="15"/>
-        <v>6267</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
@@ -1957,8 +2972,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1978,28 +2993,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
-      <c r="N1" s="38"/>
-      <c r="O1" s="38"/>
-      <c r="P1" s="38"/>
-      <c r="Q1" s="38"/>
-      <c r="R1" s="38"/>
-      <c r="S1" s="38"/>
-      <c r="T1" s="38"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+      <c r="R1" s="39"/>
+      <c r="S1" s="39"/>
+      <c r="T1" s="39"/>
       <c r="U1" s="1"/>
       <c r="V1" s="1"/>
       <c r="W1" s="1"/>
@@ -2014,16 +3029,16 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="37" t="s">
+      <c r="G2" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
-      <c r="K2" s="37"/>
-      <c r="L2" s="37"/>
-      <c r="M2" s="37"/>
-      <c r="N2" s="37"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="38"/>
+      <c r="M2" s="38"/>
+      <c r="N2" s="38"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
@@ -2068,7 +3083,7 @@
       </c>
       <c r="E6" s="3">
         <f ca="1">TODAY()</f>
-        <v>45887</v>
+        <v>46086</v>
       </c>
       <c r="F6">
         <f>YEAR(D6)</f>
@@ -2088,11 +3103,11 @@
       </c>
       <c r="K6">
         <f ca="1">DATEDIF(D6,E6,"M")</f>
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="L6">
         <f ca="1">DATEDIF(D6,E6,"D")</f>
-        <v>1123</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
@@ -2110,7 +3125,7 @@
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B10" s="4">
         <f ca="1">NOW()</f>
-        <v>45887.633442361112</v>
+        <v>46086.53264675926</v>
       </c>
       <c r="D10" s="3"/>
       <c r="I10" s="20"/>
@@ -2206,8 +3221,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AA34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2240,66 +3255,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
-      <c r="N1" s="38"/>
-      <c r="O1" s="38"/>
-      <c r="P1" s="38"/>
-      <c r="Q1" s="38"/>
-      <c r="R1" s="38"/>
-      <c r="S1" s="38"/>
-      <c r="T1" s="38"/>
-      <c r="U1" s="38"/>
-      <c r="V1" s="38"/>
-      <c r="W1" s="38"/>
-      <c r="X1" s="38"/>
-      <c r="Y1" s="38"/>
-      <c r="Z1" s="38"/>
-      <c r="AA1" s="38"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+      <c r="R1" s="39"/>
+      <c r="S1" s="39"/>
+      <c r="T1" s="39"/>
+      <c r="U1" s="39"/>
+      <c r="V1" s="39"/>
+      <c r="W1" s="39"/>
+      <c r="X1" s="39"/>
+      <c r="Y1" s="39"/>
+      <c r="Z1" s="39"/>
+      <c r="AA1" s="39"/>
     </row>
     <row r="2" spans="1:27" ht="79.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="40"/>
-      <c r="M2" s="40"/>
-      <c r="N2" s="40"/>
-      <c r="O2" s="40"/>
-      <c r="P2" s="40"/>
-      <c r="Q2" s="40"/>
-      <c r="R2" s="40"/>
-      <c r="S2" s="40"/>
-      <c r="T2" s="40"/>
-      <c r="U2" s="40"/>
-      <c r="V2" s="40"/>
-      <c r="W2" s="40"/>
-      <c r="X2" s="40"/>
-      <c r="Y2" s="40"/>
-      <c r="Z2" s="40"/>
-      <c r="AA2" s="41"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
+      <c r="Q2" s="41"/>
+      <c r="R2" s="41"/>
+      <c r="S2" s="41"/>
+      <c r="T2" s="41"/>
+      <c r="U2" s="41"/>
+      <c r="V2" s="41"/>
+      <c r="W2" s="41"/>
+      <c r="X2" s="41"/>
+      <c r="Y2" s="41"/>
+      <c r="Z2" s="41"/>
+      <c r="AA2" s="42"/>
     </row>
     <row r="3" spans="1:27" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
@@ -2468,7 +3483,7 @@
       </c>
       <c r="Z4" t="str">
         <f ca="1">UPPER(CONCATENATE("CUST",LEFT(A4,2),"BR",B4,"LOC",LEFT(C4,3),RANDBETWEEN(1000,9999)))</f>
-        <v>CUST75BRALOCTRI4822</v>
+        <v>CUST75BRALOCTRI1423</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
@@ -2520,7 +3535,7 @@
       </c>
       <c r="Z5" t="str">
         <f t="shared" ref="Z5:Z34" ca="1" si="2">UPPER(CONCATENATE("CUST",LEFT(A5,2),"BR",B5,"LOC",LEFT(C5,3),RANDBETWEEN(1000,9999)))</f>
-        <v>CUST22BRCLOCCHE3042</v>
+        <v>CUST22BRCLOCCHE3507</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
@@ -2568,7 +3583,7 @@
       </c>
       <c r="Z6" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST63BRALOCTRI8099</v>
+        <v>CUST63BRALOCTRI5621</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
@@ -2616,7 +3631,7 @@
       </c>
       <c r="Z7" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST12BRALOCTRI3011</v>
+        <v>CUST12BRALOCTRI1556</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
@@ -2664,7 +3679,7 @@
       </c>
       <c r="Z8" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST37BRALOCTRI9811</v>
+        <v>CUST37BRALOCTRI9143</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
@@ -2719,7 +3734,7 @@
       </c>
       <c r="Z9" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST69BRCLOCCHE5602</v>
+        <v>CUST69BRCLOCCHE7103</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
@@ -2767,7 +3782,7 @@
       </c>
       <c r="Z10" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST35BRALOCTRI5242</v>
+        <v>CUST35BRALOCTRI7241</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
@@ -2815,7 +3830,7 @@
       </c>
       <c r="Z11" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST31BRCLOCCHE1208</v>
+        <v>CUST31BRCLOCCHE2748</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
@@ -2863,7 +3878,7 @@
       </c>
       <c r="Z12" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST66BRALOCTRI2340</v>
+        <v>CUST66BRALOCTRI1382</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
@@ -2911,7 +3926,7 @@
       </c>
       <c r="Z13" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST69BRBLOCKAR7286</v>
+        <v>CUST69BRBLOCKAR3086</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
@@ -2959,7 +3974,7 @@
       </c>
       <c r="Z14" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST35BRBLOCKAR2229</v>
+        <v>CUST35BRBLOCKAR8641</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
@@ -3007,7 +4022,7 @@
       </c>
       <c r="Z15" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST52BRBLOCKAR3344</v>
+        <v>CUST52BRBLOCKAR4282</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
@@ -3055,7 +4070,7 @@
       </c>
       <c r="Z16" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST36BRALOCTRI2964</v>
+        <v>CUST36BRALOCTRI1614</v>
       </c>
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.25">
@@ -3103,7 +4118,7 @@
       </c>
       <c r="Z17" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST25BRALOCTRI9593</v>
+        <v>CUST25BRALOCTRI7696</v>
       </c>
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.25">
@@ -3151,7 +4166,7 @@
       </c>
       <c r="Z18" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST82BRALOCTRI7610</v>
+        <v>CUST82BRALOCTRI8728</v>
       </c>
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.25">
@@ -3199,7 +4214,7 @@
       </c>
       <c r="Z19" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST29BRBLOCKAR4488</v>
+        <v>CUST29BRBLOCKAR6855</v>
       </c>
     </row>
     <row r="20" spans="1:26" x14ac:dyDescent="0.25">
@@ -3247,7 +4262,7 @@
       </c>
       <c r="Z20" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST65BRALOCTRI7116</v>
+        <v>CUST65BRALOCTRI7510</v>
       </c>
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.25">
@@ -3295,7 +4310,7 @@
       </c>
       <c r="Z21" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST76BRALOCTRI1880</v>
+        <v>CUST76BRALOCTRI1286</v>
       </c>
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.25">
@@ -3343,7 +4358,7 @@
       </c>
       <c r="Z22" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST32BRALOCTRI9684</v>
+        <v>CUST32BRALOCTRI2869</v>
       </c>
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.25">
@@ -3391,7 +4406,7 @@
       </c>
       <c r="Z23" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST31BRBLOCKAR1751</v>
+        <v>CUST31BRBLOCKAR4553</v>
       </c>
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.25">
@@ -3439,7 +4454,7 @@
       </c>
       <c r="Z24" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST30BRCLOCCHE5564</v>
+        <v>CUST30BRCLOCCHE9240</v>
       </c>
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.25">
@@ -3487,7 +4502,7 @@
       </c>
       <c r="Z25" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST37BRBLOCKAR1425</v>
+        <v>CUST37BRBLOCKAR6218</v>
       </c>
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.25">
@@ -3535,7 +4550,7 @@
       </c>
       <c r="Z26" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST27BRBLOCKAR1869</v>
+        <v>CUST27BRBLOCKAR7161</v>
       </c>
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.25">
@@ -3583,7 +4598,7 @@
       </c>
       <c r="Z27" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST63BRALOCTRI6900</v>
+        <v>CUST63BRALOCTRI3608</v>
       </c>
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.25">
@@ -3631,7 +4646,7 @@
       </c>
       <c r="Z28" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST54BRALOCTRI6481</v>
+        <v>CUST54BRALOCTRI3969</v>
       </c>
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.25">
@@ -3679,7 +4694,7 @@
       </c>
       <c r="Z29" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST22BRALOCTRI9273</v>
+        <v>CUST22BRALOCTRI6562</v>
       </c>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
@@ -3727,7 +4742,7 @@
       </c>
       <c r="Z30" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST64BRBLOCKAR2574</v>
+        <v>CUST64BRBLOCKAR4209</v>
       </c>
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.25">
@@ -3775,7 +4790,7 @@
       </c>
       <c r="Z31" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST18BRALOCTRI2934</v>
+        <v>CUST18BRALOCTRI5890</v>
       </c>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
@@ -3823,7 +4838,7 @@
       </c>
       <c r="Z32" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST14BRBLOCKAR9979</v>
+        <v>CUST14BRBLOCKAR9494</v>
       </c>
     </row>
     <row r="33" spans="1:26" x14ac:dyDescent="0.25">
@@ -3871,7 +4886,7 @@
       </c>
       <c r="Z33" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST84BRALOCTRI6151</v>
+        <v>CUST84BRALOCTRI5792</v>
       </c>
     </row>
     <row r="34" spans="1:26" x14ac:dyDescent="0.25">
@@ -3919,7 +4934,7 @@
       </c>
       <c r="Z34" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>CUST87BRBLOCKAR6552</v>
+        <v>CUST87BRBLOCKAR6447</v>
       </c>
     </row>
   </sheetData>
@@ -3932,8 +4947,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:U14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3957,13 +4972,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>192</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="43" t="s">
         <v>199</v>
       </c>
-      <c r="D1" s="42" t="s">
+      <c r="D1" s="43" t="s">
         <v>200</v>
       </c>
       <c r="E1" s="7" t="s">
@@ -4010,12 +5025,12 @@
       </c>
     </row>
     <row r="2" spans="1:21" ht="83.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42"/>
-      <c r="B2" s="43" t="s">
+      <c r="A2" s="43"/>
+      <c r="B2" s="44" t="s">
         <v>193</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
       <c r="E2" s="7" t="s">
         <v>79</v>
       </c>
@@ -4060,10 +5075,10 @@
       </c>
     </row>
     <row r="3" spans="1:21" ht="67.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="42"/>
-      <c r="B3" s="43"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
+      <c r="A3" s="43"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
       <c r="E3" s="9" t="s">
         <v>90</v>
       </c>
@@ -4476,8 +5491,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:T17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4495,664 +5510,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="48" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="47"/>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="47"/>
-      <c r="O1" s="47"/>
-      <c r="P1" s="47"/>
-      <c r="Q1" s="47"/>
-      <c r="R1" s="47"/>
-      <c r="S1" s="47"/>
-      <c r="T1" s="47"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
-        <v>65</v>
-      </c>
-      <c r="B2" s="42" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="42" t="s">
-        <v>67</v>
-      </c>
-      <c r="E2" s="45" t="s">
-        <v>109</v>
-      </c>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="46"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="42"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="21"/>
-      <c r="P3" s="21"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A4" s="42"/>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="G4" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="H4" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="I4" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="J4" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="K4" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="L4" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="M4" s="23" t="s">
-        <v>126</v>
-      </c>
-      <c r="N4" s="23" t="s">
-        <v>127</v>
-      </c>
-      <c r="O4" s="21"/>
-      <c r="P4" s="21"/>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A5" s="12">
-        <v>44</v>
-      </c>
-      <c r="B5" s="12">
-        <v>0</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5">
-        <f>AVERAGE(A5:A9)</f>
-        <v>35.6</v>
-      </c>
-      <c r="E5">
-        <f>MEDIAN(A5:A9)</f>
-        <v>30</v>
-      </c>
-      <c r="F5">
-        <f>MODE(A5:A9)</f>
-        <v>30</v>
-      </c>
-      <c r="G5">
-        <f>COUNT(A5:A9)</f>
-        <v>5</v>
-      </c>
-      <c r="H5">
-        <f>COUNTA(C5:C9)</f>
-        <v>5</v>
-      </c>
-      <c r="I5">
-        <f>COUNTIF(C5:C9,"A")</f>
-        <v>3</v>
-      </c>
-      <c r="J5">
-        <f>COUNTIFS(C5:C9,"A",B5:B9,0)</f>
-        <v>2</v>
-      </c>
-      <c r="K5">
-        <f>MAX(B5:B9)</f>
-        <v>55</v>
-      </c>
-      <c r="L5">
-        <f>MIN(B5:B9)</f>
-        <v>0</v>
-      </c>
-      <c r="M5" s="21">
-        <f>STDEV(A5:A9)</f>
-        <v>7.6681158050723228</v>
-      </c>
-      <c r="N5">
-        <f>VAR(A5:A9)</f>
-        <v>58.799999999999955</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
-        <v>30</v>
-      </c>
-      <c r="B6" s="12">
-        <v>25</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6">
-        <f t="shared" ref="D6:D9" si="0">AVERAGE(A6:A10)</f>
-        <v>33.5</v>
-      </c>
-      <c r="E6">
-        <f t="shared" ref="E6:E9" si="1">MEDIAN(A6:A10)</f>
-        <v>30</v>
-      </c>
-      <c r="F6">
-        <f>MODE(A5:A10)</f>
-        <v>30</v>
-      </c>
-      <c r="G6">
-        <f t="shared" ref="G6:G9" si="2">COUNT(A6:A10)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
-        <v>30</v>
-      </c>
-      <c r="B7" s="12">
-        <v>0</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7">
-        <f t="shared" si="0"/>
-        <v>34.666666666666664</v>
-      </c>
-      <c r="E7">
-        <f t="shared" si="1"/>
-        <v>30</v>
-      </c>
-      <c r="G7">
-        <f t="shared" si="2"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
-        <v>30</v>
-      </c>
-      <c r="B8" s="12">
-        <v>45</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8">
-        <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-      <c r="E8">
-        <f t="shared" si="1"/>
-        <v>37</v>
-      </c>
-      <c r="G8">
-        <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A9" s="12">
-        <v>44</v>
-      </c>
-      <c r="B9" s="12">
-        <v>55</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-      <c r="E9">
-        <f t="shared" si="1"/>
-        <v>44</v>
-      </c>
-      <c r="G9">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="N11">
-        <f>SQRT(N5)</f>
-        <v>7.6681158050723228</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="H15" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A16" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="B16" s="44"/>
-      <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16">
-        <v>3</v>
-      </c>
-      <c r="E16">
-        <v>4</v>
-      </c>
-      <c r="F16">
-        <v>5</v>
-      </c>
-      <c r="G16">
-        <v>3</v>
-      </c>
-      <c r="H16">
-        <f>MEDIAN(C16:G16)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="44" t="s">
-        <v>117</v>
-      </c>
-      <c r="B17" s="44"/>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17">
-        <v>3</v>
-      </c>
-      <c r="E17">
-        <v>3</v>
-      </c>
-      <c r="F17">
-        <v>4</v>
-      </c>
-      <c r="G17">
-        <v>5</v>
-      </c>
-      <c r="H17">
-        <v>3</v>
-      </c>
-      <c r="I17" t="s">
-        <v>119</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="E2:P2"/>
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C2:C4"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:T21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:20" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="B1" s="47" t="s">
-        <v>112</v>
-      </c>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="47"/>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="47"/>
-      <c r="O1" s="47"/>
-      <c r="P1" s="47"/>
-      <c r="Q1" s="47"/>
-      <c r="R1" s="47"/>
-      <c r="S1" s="47"/>
-      <c r="T1" s="47"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="42" t="s">
-        <v>65</v>
-      </c>
-      <c r="C2" s="42" t="s">
-        <v>133</v>
-      </c>
-      <c r="D2" s="45" t="s">
-        <v>111</v>
-      </c>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="42"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A4" s="42"/>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="12">
-        <v>40</v>
-      </c>
-      <c r="C5" s="12">
-        <v>0</v>
-      </c>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="12">
-        <v>55</v>
-      </c>
-      <c r="C6" s="12">
-        <v>55</v>
-      </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="H6" s="25" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="B7" s="12">
-        <v>30</v>
-      </c>
-      <c r="C7" s="12">
-        <v>0</v>
-      </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="24">
-        <f>VLOOKUP(G7,A5:F9,3)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="B8" s="12">
-        <v>40</v>
-      </c>
-      <c r="C8" s="12">
-        <v>45</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="E8" s="12">
-        <v>33</v>
-      </c>
-      <c r="F8" s="12">
-        <v>333</v>
-      </c>
-      <c r="G8" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" s="24">
-        <f>VLOOKUP(G8,A5:F9,3)</f>
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="B9" s="12">
-        <v>50</v>
-      </c>
-      <c r="C9" s="12">
-        <v>55</v>
-      </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="24" t="s">
-        <v>130</v>
-      </c>
-      <c r="H9" s="24">
-        <f>VLOOKUP(G9,A5:F9,3)</f>
-        <v>55</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="H15" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A16" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="G16" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="H16" s="26" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="B17" s="12">
-        <v>40</v>
-      </c>
-      <c r="C17" s="12">
-        <v>55</v>
-      </c>
-      <c r="D17" s="12">
-        <v>30</v>
-      </c>
-      <c r="E17" s="12">
-        <v>40</v>
-      </c>
-      <c r="F17" s="12">
-        <v>50</v>
-      </c>
-      <c r="G17" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="H17" s="25">
-        <f>HLOOKUP(G17,A16:F26,2,)</f>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="B18" s="12">
-        <v>0</v>
-      </c>
-      <c r="C18" s="12">
-        <v>25</v>
-      </c>
-      <c r="D18" s="12">
-        <v>0</v>
-      </c>
-      <c r="E18" s="12">
-        <v>45</v>
-      </c>
-      <c r="F18" s="12">
-        <v>55</v>
-      </c>
-      <c r="G18" s="24">
-        <v>50</v>
-      </c>
-      <c r="H18" s="25">
-        <f>HLOOKUP(G18,B17:F21,2,TRUE)</f>
-        <v>55</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="F19" s="12"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12">
-        <v>33</v>
-      </c>
-      <c r="F20" s="12"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12">
-        <v>333</v>
-      </c>
-      <c r="F21" s="12"/>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="D2:N2"/>
-    <mergeCell ref="B1:T1"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="A2:A4"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:S15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="18.85546875" customWidth="1"/>
-    <col min="5" max="5" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:19" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="C1" s="48" t="s">
-        <v>150</v>
-      </c>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
       <c r="D1" s="48"/>
       <c r="E1" s="48"/>
       <c r="F1" s="48"/>
@@ -5169,23 +5531,676 @@
       <c r="Q1" s="48"/>
       <c r="R1" s="48"/>
       <c r="S1" s="48"/>
+      <c r="T1" s="48"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A2" s="43" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
+      <c r="P2" s="47"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A3" s="43"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="F4" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="H4" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="I4" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="J4" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="K4" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="L4" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="M4" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="N4" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>44</v>
+      </c>
+      <c r="B5" s="12">
+        <v>0</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <f>AVERAGE(A5:A9)</f>
+        <v>35.6</v>
+      </c>
+      <c r="E5">
+        <f>MEDIAN(A5:A9)</f>
+        <v>30</v>
+      </c>
+      <c r="F5">
+        <f>MODE(A5:A9)</f>
+        <v>30</v>
+      </c>
+      <c r="G5">
+        <f>COUNT(A5:A9)</f>
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <f>COUNTA(C5:C9)</f>
+        <v>5</v>
+      </c>
+      <c r="I5">
+        <f>COUNTIF(C5:C9,"A")</f>
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <f>COUNTIFS(C5:C9,"A",B5:B9,0)</f>
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <f>MAX(B5:B9)</f>
+        <v>55</v>
+      </c>
+      <c r="L5">
+        <f>MIN(B5:B9)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="21">
+        <f>STDEV(A5:A9)</f>
+        <v>7.6681158050723228</v>
+      </c>
+      <c r="N5">
+        <f>VAR(A5:A9)</f>
+        <v>58.799999999999955</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>30</v>
+      </c>
+      <c r="B6" s="12">
+        <v>25</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6">
+        <f t="shared" ref="D6:D9" si="0">AVERAGE(A6:A10)</f>
+        <v>33.5</v>
+      </c>
+      <c r="E6">
+        <f t="shared" ref="E6:E9" si="1">MEDIAN(A6:A10)</f>
+        <v>30</v>
+      </c>
+      <c r="F6">
+        <f>MODE(A5:A10)</f>
+        <v>30</v>
+      </c>
+      <c r="G6">
+        <f t="shared" ref="G6:G9" si="2">COUNT(A6:A10)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>30</v>
+      </c>
+      <c r="B7" s="12">
+        <v>0</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>34.666666666666664</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A8" s="12">
+        <v>30</v>
+      </c>
+      <c r="B8" s="12">
+        <v>45</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A9" s="12">
+        <v>44</v>
+      </c>
+      <c r="B9" s="12">
+        <v>55</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>44</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="N11">
+        <f>SQRT(N5)</f>
+        <v>7.6681158050723228</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="H15" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A16" s="45" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" s="45"/>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>4</v>
+      </c>
+      <c r="F16">
+        <v>5</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
+        <f>MEDIAN(C16:G16)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="45" t="s">
+        <v>117</v>
+      </c>
+      <c r="B17" s="45"/>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>4</v>
+      </c>
+      <c r="G17">
+        <v>5</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="E2:P2"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:T21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="48" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
+      <c r="P1" s="48"/>
+      <c r="Q1" s="48"/>
+      <c r="R1" s="48"/>
+      <c r="S1" s="48"/>
+      <c r="T1" s="48"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A2" s="43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="43" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2" s="46" t="s">
+        <v>111</v>
+      </c>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A3" s="43"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A4" s="43"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="12">
+        <v>40</v>
+      </c>
+      <c r="C5" s="12">
+        <v>0</v>
+      </c>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="12">
+        <v>55</v>
+      </c>
+      <c r="C6" s="12">
+        <v>55</v>
+      </c>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="H6" s="25" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" s="12">
+        <v>30</v>
+      </c>
+      <c r="C7" s="12">
+        <v>0</v>
+      </c>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="24">
+        <f>VLOOKUP(G7,A5:F9,3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" s="12">
+        <v>40</v>
+      </c>
+      <c r="C8" s="12">
+        <v>45</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" s="12">
+        <v>33</v>
+      </c>
+      <c r="F8" s="12">
+        <v>333</v>
+      </c>
+      <c r="G8" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" s="24">
+        <f>VLOOKUP(G8,A5:F9,3)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="B9" s="12">
+        <v>50</v>
+      </c>
+      <c r="C9" s="12">
+        <v>55</v>
+      </c>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="H9" s="24">
+        <f>VLOOKUP(G9,A5:F9,3)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="H15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A16" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="G16" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="H16" s="26" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="12">
+        <v>40</v>
+      </c>
+      <c r="C17" s="12">
+        <v>55</v>
+      </c>
+      <c r="D17" s="12">
+        <v>30</v>
+      </c>
+      <c r="E17" s="12">
+        <v>40</v>
+      </c>
+      <c r="F17" s="12">
+        <v>50</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="H17" s="25">
+        <f>HLOOKUP(G17,A16:F26,2,)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="B18" s="12">
+        <v>0</v>
+      </c>
+      <c r="C18" s="12">
+        <v>25</v>
+      </c>
+      <c r="D18" s="12">
+        <v>0</v>
+      </c>
+      <c r="E18" s="12">
+        <v>45</v>
+      </c>
+      <c r="F18" s="12">
+        <v>55</v>
+      </c>
+      <c r="G18" s="24">
+        <v>50</v>
+      </c>
+      <c r="H18" s="25">
+        <f>HLOOKUP(G18,B17:F21,2,TRUE)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="F19" s="12"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12">
+        <v>33</v>
+      </c>
+      <c r="F20" s="12"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12">
+        <v>333</v>
+      </c>
+      <c r="F21" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="D2:N2"/>
+    <mergeCell ref="B1:T1"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="A2:A4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="5" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="C1" s="49" t="s">
+        <v>150</v>
+      </c>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="49"/>
+      <c r="J1" s="49"/>
+      <c r="K1" s="49"/>
+      <c r="L1" s="49"/>
+      <c r="M1" s="49"/>
+      <c r="N1" s="49"/>
+      <c r="O1" s="49"/>
+      <c r="P1" s="49"/>
+      <c r="Q1" s="49"/>
+      <c r="R1" s="49"/>
+      <c r="S1" s="49"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="45" t="s">
         <v>158</v>
       </c>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="L2" s="44"/>
-      <c r="M2" s="44"/>
-      <c r="N2" s="44"/>
-      <c r="O2" s="44"/>
-      <c r="P2" s="44"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="28" t="s">
@@ -5313,124 +6328,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="str">
-        <f>'Reference Functions'!A4</f>
-        <v>Name</v>
-      </c>
-      <c r="B1" t="str">
-        <f>'Reference Functions'!C4</f>
-        <v>Gender</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="str">
-        <f>'Reference Functions'!A5</f>
-        <v>John</v>
-      </c>
-      <c r="B2" t="str">
-        <f>'Reference Functions'!C5</f>
-        <v>Male</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="str">
-        <f>'Reference Functions'!A6</f>
-        <v>Sarah</v>
-      </c>
-      <c r="B3" t="str">
-        <f>'Reference Functions'!C6</f>
-        <v>Female</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="str">
-        <f>'Reference Functions'!A7</f>
-        <v>Mike</v>
-      </c>
-      <c r="B4" t="str">
-        <f>'Reference Functions'!C7</f>
-        <v>male</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <f>'Reference Functions'!A8</f>
-        <v>0</v>
-      </c>
-      <c r="B5">
-        <f>'Reference Functions'!C8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <f>'Reference Functions'!A9</f>
-        <v>0</v>
-      </c>
-      <c r="B6">
-        <f>'Reference Functions'!C9</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <f>'Reference Functions'!A10</f>
-        <v>0</v>
-      </c>
-      <c r="B7">
-        <f>'Reference Functions'!C10</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <f>'Reference Functions'!A11</f>
-        <v>0</v>
-      </c>
-      <c r="B8">
-        <f>'Reference Functions'!C11</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <f>'Reference Functions'!A12</f>
-        <v>0</v>
-      </c>
-      <c r="B9">
-        <f>'Reference Functions'!C12</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <f>'Reference Functions'!A13</f>
-        <v>0</v>
-      </c>
-      <c r="B10">
-        <f>'Reference Functions'!C13</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <f>'Reference Functions'!A14</f>
-        <v>0</v>
-      </c>
-      <c r="B11">
-        <f>'Reference Functions'!C14</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>